<commit_message>
subiendo cambios y actualizaciones
</commit_message>
<xml_diff>
--- a/maparuta.xlsx
+++ b/maparuta.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santiago\OneDrive\Escritorio\DecimoSemestre\IA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santiago\OneDrive\Escritorio\Repositorios\route-map-IA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99F965F8-56DB-4D91-B8DE-0D0BB3AA0771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DBD0DF-A4CA-496F-9526-C9B323C4A085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{41B2DF8D-D692-4519-963C-2F8D1AF66B97}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Comprension del Negocio</t>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t>Comprension de los datos</t>
-  </si>
-  <si>
-    <t>Limpieza de los datos</t>
   </si>
   <si>
     <t>Mapa de Ruta (DataSet del Titanic)</t>
@@ -69,6 +66,116 @@
       </rPr>
       <t>Es ver las primeras filas de una tabla de datos para tener una idea rápida de su contenido y estructura sin abrir el archivo completo.</t>
     </r>
+  </si>
+  <si>
+    <t>Limpieza y feature engineering</t>
+  </si>
+  <si>
+    <t>Identifica si hay nulos isnull
+X_completo_training.isnull()</t>
+  </si>
+  <si>
+    <t>Borrar nulos dropna
+#X_completo_training =  X_completo_training.dropna()
+#X_completo_training</t>
+  </si>
+  <si>
+    <t>Limpiar columnas numericas, Rellenar vacios por media de la misma clase</t>
+  </si>
+  <si>
+    <t>Limpiar columnas categoricas, rellenar vacios por moda de la misma clase</t>
+  </si>
+  <si>
+    <t>Matriz de correlacion de Pearson- etapa de comprensión de los datos</t>
+  </si>
+  <si>
+    <t>Eliminar columnas</t>
+  </si>
+  <si>
+    <t>Modelamiento y evaluación</t>
+  </si>
+  <si>
+    <t>Decision Tree classifer
+# Create Decision Tree classifer object
+#verificar si usa Gini o usa entropia
+clf = DecisionTreeClassifier(criterion='entropy')
+# Train Decision Tree Classifer
+clf = clf.fit(X_train_res,y_train_res)</t>
+  </si>
+  <si>
+    <t>Calcular la importancia de cada atributo con arbol de decisión
+feature_cols = X_train_res.columns
+# se obtiene la importancia de cada atributo a partir del arbol
+print("for para calcular la importancia de cada atributo")
+# se crea un diccionario
+diccionario = {}
+# tree.feature_importances_ se obtiene la importancia de cada atributo
+#zip  devuelve un iterador de tuplas basado en los objetos iterables
+for name, importance in zip(feature_cols, clf.feature_importances_):
+    diccionario[name] = importance
+import operator
+sortedDict = sorted(diccionario.items(), key=operator.itemgetter(1))
+sortedDict</t>
+  </si>
+  <si>
+    <t>Matriz de confusión
+# matriz de confusion
+from sklearn.metrics import confusion_matrix
+print(confusion_matrix(y_test_res, y_pred))</t>
+  </si>
+  <si>
+    <t>Validación cruzada
+# se efectúa validación cruzada
+from sklearn import model_selection
+kFold = model_selection.KFold(n_splits=10)
+scoring = 'accuracy'
+puntaje= (model_selection.cross_val_score(clf, X_train, y_train,  scoring = scoring, cv = kFold))
+print (f"( {puntaje.mean()}, {puntaje.std()}")</t>
+  </si>
+  <si>
+    <t>classification_report
+from sklearn.metrics import classification_report
+print(classification_report(y_test_res, y_pred))</t>
+  </si>
+  <si>
+    <t>Ajuste de hiperparámetros</t>
+  </si>
+  <si>
+    <t>Bayes</t>
+  </si>
+  <si>
+    <t>Decision Tree classifer
+from sklearn.feature_selection import SelectKBest
+from sklearn.naive_bayes import GaussianNB
+#X = df.drop('sobreviviente', axis=1)
+#Y = df['sobreviviente']
+#este es un metodo de seleccion de caracteristicas
+#le da puntaje a cada caracteristica y borra todas las demas
+#excepto las que tienen puntaje mas alto
+best=SelectKBest(k=5)
+print (y)
+X_new = best.fit_transform(X_completo_training, y_train)
+selected = best.get_support(indices=True)
+print(selected)
+caracteristicasUsadas =X_completo_training.columns[selected]
+print(caracteristicasUsadas)
+# Split dataset in training and test datasets
+#X_train, X_test, y_train, y_test = train_test_split(X, y, test_size=0.3, random_state=1)
+gnb = GaussianNB()
+# Train classifier
+gnb.fit(X_completo_training[caracteristicasUsadas].values, y_train)
+#se predice con las variables seleccionadas
+y_pred = gnb.predict(X_completo_test[caracteristicasUsadas])
+ #Devuelve la precisión media en los datos y etiquetas de prueba dados.
+print('Precision con el set de prueba: {:.2f}'.format(gnb.score(X_completo_test[caracteristicasUsadas], y_test)))
+print('Se obtiene la precision con el dataset de entrenamiento: {:.2f}'.format(gnb.score(X_completo_training[caracteristicasUsadas], y_train)))
+puntaje = calcular_validacion_cruzada(gnb, X_completo_training, y_train)
+print ("validacion cruzada")
+print (f"( {puntaje.mean()}, {puntaje.std()} )")
+#                 ['ingresos', 'ahorros', 'hijos', 'trabajo', 'financiar']
+print("se hace prediccion")
+print(gnb.predict([[1000,        4000,     1,       6,         100000]]))
+#Resultado esperado 0-Alquilar, 1-Comprar casa</t>
   </si>
 </sst>
 </file>
@@ -96,12 +203,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="18"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -117,6 +218,13 @@
     <font>
       <sz val="12"/>
       <color rgb="FFA20000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -236,58 +344,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -786,201 +897,323 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{061E4B78-CCD8-4166-8919-8D3B984C7257}">
-  <dimension ref="B1:S18"/>
+  <dimension ref="B1:AE18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="11" max="11" width="16.5703125" customWidth="1"/>
     <col min="12" max="12" width="20.28515625" customWidth="1"/>
     <col min="13" max="13" width="18.85546875" customWidth="1"/>
     <col min="14" max="14" width="38" customWidth="1"/>
+    <col min="17" max="17" width="15.5703125" customWidth="1"/>
+    <col min="18" max="18" width="18.140625" customWidth="1"/>
+    <col min="24" max="24" width="19.28515625" customWidth="1"/>
+    <col min="30" max="30" width="20.7109375" customWidth="1"/>
+    <col min="31" max="31" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="14"/>
+    </row>
+    <row r="3" spans="2:31" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D3" s="15"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="17"/>
+    </row>
+    <row r="6" spans="2:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="2:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="6"/>
+      <c r="E7" s="7"/>
+      <c r="K7" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="L7" s="6"/>
+      <c r="M7" s="7"/>
+      <c r="Q7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="R7" s="6"/>
+      <c r="S7" s="7"/>
+      <c r="W7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="7"/>
+      <c r="AC7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD7" s="6"/>
+      <c r="AE7" s="7"/>
+    </row>
+    <row r="8" spans="2:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="8"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="10"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="10"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="10"/>
+      <c r="W8" s="8"/>
+      <c r="X8" s="9"/>
+      <c r="Y8" s="10"/>
+      <c r="AC8" s="8"/>
+      <c r="AD8" s="9"/>
+      <c r="AE8" s="10"/>
+    </row>
+    <row r="9" spans="2:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="8"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="10"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="10"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="10"/>
+      <c r="W9" s="8"/>
+      <c r="X9" s="9"/>
+      <c r="Y9" s="10"/>
+      <c r="AC9" s="8"/>
+      <c r="AD9" s="9"/>
+      <c r="AE9" s="10"/>
+    </row>
+    <row r="10" spans="2:31" ht="190.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="4"/>
-    </row>
-    <row r="3" spans="2:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="5"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="7"/>
-    </row>
-    <row r="6" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="D7" s="9"/>
-      <c r="E7" s="10"/>
-      <c r="K7" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="L7" s="9"/>
-      <c r="M7" s="10"/>
-      <c r="Q7" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="R7" s="9"/>
-      <c r="S7" s="10"/>
-    </row>
-    <row r="8" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="11"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="13"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="13"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="12"/>
-      <c r="S8" s="13"/>
-    </row>
-    <row r="9" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="13"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="13"/>
-      <c r="Q9" s="11"/>
-      <c r="R9" s="12"/>
-      <c r="S9" s="13"/>
-    </row>
-    <row r="10" spans="2:19" ht="144" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="17" t="s">
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="K10" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="K10" s="17" t="s">
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="2"/>
+      <c r="Q10" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="R10" s="11"/>
+      <c r="S10" s="11"/>
+      <c r="W10" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="X10" s="11"/>
+      <c r="Y10" s="11"/>
+      <c r="AC10" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="AD10" s="19"/>
+      <c r="AE10" s="19"/>
+    </row>
+    <row r="11" spans="2:31" ht="285.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="K11" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="18"/>
-      <c r="Q10" s="16"/>
-      <c r="R10" s="16"/>
-      <c r="S10" s="16"/>
-    </row>
-    <row r="11" spans="2:19" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="17" t="s">
-        <v>1</v>
-      </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="K11" s="17" t="s">
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="Q11" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="R11" s="11"/>
+      <c r="S11" s="11"/>
+      <c r="W11" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="X11" s="11"/>
+      <c r="Y11" s="11"/>
+      <c r="AC11" s="11"/>
+      <c r="AD11" s="11"/>
+      <c r="AE11" s="11"/>
+    </row>
+    <row r="12" spans="2:31" ht="135.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="K12" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="Q11" s="14"/>
-      <c r="R11" s="14"/>
-      <c r="S11" s="14"/>
-    </row>
-    <row r="12" spans="2:19" ht="135.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="K12" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
-      <c r="Q12" s="14"/>
-      <c r="R12" s="14"/>
-      <c r="S12" s="14"/>
-    </row>
-    <row r="13" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="14"/>
-      <c r="M13" s="14"/>
-      <c r="Q13" s="14"/>
-      <c r="R13" s="14"/>
-      <c r="S13" s="14"/>
-    </row>
-    <row r="14" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="14"/>
-      <c r="Q14" s="14"/>
-      <c r="R14" s="14"/>
-      <c r="S14" s="14"/>
-    </row>
-    <row r="15" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="14"/>
-      <c r="Q15" s="14"/>
-      <c r="R15" s="14"/>
-      <c r="S15" s="14"/>
-    </row>
-    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="15"/>
-      <c r="M16" s="15"/>
-      <c r="Q16" s="15"/>
-      <c r="R16" s="15"/>
-      <c r="S16" s="15"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="Q12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="R12" s="3"/>
+      <c r="S12" s="3"/>
+      <c r="W12" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="X12" s="3"/>
+      <c r="Y12" s="3"/>
+      <c r="AC12" s="11"/>
+      <c r="AD12" s="3"/>
+      <c r="AE12" s="3"/>
+    </row>
+    <row r="13" spans="2:31" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="Q13" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="R13" s="11"/>
+      <c r="S13" s="11"/>
+      <c r="W13" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="X13" s="11"/>
+      <c r="Y13" s="11"/>
+      <c r="AC13" s="11"/>
+      <c r="AD13" s="11"/>
+      <c r="AE13" s="11"/>
+    </row>
+    <row r="14" spans="2:31" ht="179.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="Q14" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="R14" s="11"/>
+      <c r="S14" s="11"/>
+      <c r="W14" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="X14" s="11"/>
+      <c r="Y14" s="11"/>
+      <c r="AC14" s="11"/>
+      <c r="AD14" s="11"/>
+      <c r="AE14" s="11"/>
+    </row>
+    <row r="15" spans="2:31" ht="120.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="11"/>
+      <c r="S15" s="11"/>
+      <c r="W15" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="X15" s="11"/>
+      <c r="Y15" s="11"/>
+    </row>
+    <row r="16" spans="2:31" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="Q16" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="R16" s="18"/>
+      <c r="S16" s="18"/>
     </row>
     <row r="17" spans="3:19" x14ac:dyDescent="0.25">
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="15"/>
-      <c r="M17" s="15"/>
-      <c r="Q17" s="15"/>
-      <c r="R17" s="15"/>
-      <c r="S17" s="15"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="Q17" s="4"/>
+      <c r="R17" s="4"/>
+      <c r="S17" s="4"/>
     </row>
     <row r="18" spans="3:19" x14ac:dyDescent="0.25">
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="15"/>
-      <c r="S18" s="15"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="Q18" s="4"/>
+      <c r="R18" s="4"/>
+      <c r="S18" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="44">
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="AC7:AE9"/>
+    <mergeCell ref="AC10:AE10"/>
+    <mergeCell ref="AC11:AE11"/>
+    <mergeCell ref="AC12:AE12"/>
+    <mergeCell ref="AC13:AE13"/>
+    <mergeCell ref="AC14:AE14"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="W7:Y9"/>
+    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="W11:Y11"/>
+    <mergeCell ref="W12:Y12"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="D2:P3"/>
+    <mergeCell ref="C7:E9"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="K7:M9"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="K13:M13"/>
+    <mergeCell ref="Q14:S14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="Q7:S9"/>
+    <mergeCell ref="Q10:S10"/>
+    <mergeCell ref="Q11:S11"/>
+    <mergeCell ref="Q12:S12"/>
+    <mergeCell ref="Q13:S13"/>
     <mergeCell ref="Q15:S15"/>
     <mergeCell ref="Q16:S16"/>
     <mergeCell ref="Q17:S17"/>
@@ -989,29 +1222,6 @@
     <mergeCell ref="K16:M16"/>
     <mergeCell ref="K17:M17"/>
     <mergeCell ref="K18:M18"/>
-    <mergeCell ref="Q7:S9"/>
-    <mergeCell ref="Q10:S10"/>
-    <mergeCell ref="Q11:S11"/>
-    <mergeCell ref="Q12:S12"/>
-    <mergeCell ref="Q13:S13"/>
-    <mergeCell ref="Q14:S14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="K7:M9"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="K13:M13"/>
-    <mergeCell ref="K14:M14"/>
-    <mergeCell ref="D2:P3"/>
-    <mergeCell ref="C7:E9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>